<commit_message>
fix: template com campos obrigatórios corretos (só email/telefone opcionais)
</commit_message>
<xml_diff>
--- a/docs/template_funcionarios.xlsx
+++ b/docs/template_funcionarios.xlsx
@@ -21,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="R$ #,##0.00"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -71,6 +71,11 @@
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="001e293b"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <color rgb="00475569"/>
       <sz val="10"/>
     </font>
@@ -85,7 +90,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -109,12 +114,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFE0E0"/>
+        <fgColor rgb="00FFD6D6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EDF1F7"/>
+        <fgColor rgb="00E8F4FD"/>
       </patternFill>
     </fill>
     <fill>
@@ -125,6 +130,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDF1F7"/>
       </patternFill>
     </fill>
     <fill>
@@ -192,7 +202,7 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -201,29 +211,29 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -594,13 +604,13 @@
   <dimension ref="A1:G104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28.57142857142857" customWidth="1" min="1" max="1"/>
-    <col width="31.42857142857143" customWidth="1" min="2" max="2"/>
-    <col width="18.57142857142857" customWidth="1" min="3" max="3"/>
-    <col width="25.71428571428572" customWidth="1" min="4" max="4"/>
-    <col width="18.57142857142857" customWidth="1" min="5" max="5"/>
-    <col width="17.14285714285714" customWidth="1" min="6" max="6"/>
-    <col width="15.71428571428571" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -613,11 +623,11 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>🔴 Campo obrigatório (fundo rosa)   |   ⚪ Campo opcional (fundo azul)   |   🟢 Linha de exemplo (não importar)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
+          <t>🔴 Campo obrigatório (fundo rosa)   |   🔵 Campo opcional (fundo azul)   |   🟢 Linha de exemplo (não importar)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Nome Completo *</t>
@@ -635,22 +645,22 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Cargo / Função</t>
+          <t>Cargo / Função *</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Custo por Hora (R$)</t>
+          <t>Custo por Hora (R$) *</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Horas por Dia Útil</t>
+          <t>Horas por Dia Útil *</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Ativo (SIM/NÃO)</t>
+          <t>Ativo (SIM/NÃO) *</t>
         </is>
       </c>
     </row>
@@ -687,1118 +697,1521 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="18" customHeight="1">
       <c r="A5" s="6" t="n"/>
       <c r="B5" s="7" t="n"/>
       <c r="C5" s="7" t="n"/>
-      <c r="D5" s="7" t="n"/>
+      <c r="D5" s="6" t="n"/>
       <c r="E5" s="8" t="n"/>
-      <c r="F5" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G5" s="7" t="n"/>
-    </row>
-    <row r="6">
+      <c r="F5" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
       <c r="A6" s="6" t="n"/>
       <c r="B6" s="7" t="n"/>
       <c r="C6" s="7" t="n"/>
-      <c r="D6" s="7" t="n"/>
+      <c r="D6" s="6" t="n"/>
       <c r="E6" s="8" t="n"/>
-      <c r="F6" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G6" s="7" t="n"/>
-    </row>
-    <row r="7">
+      <c r="F6" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
       <c r="A7" s="6" t="n"/>
       <c r="B7" s="7" t="n"/>
       <c r="C7" s="7" t="n"/>
-      <c r="D7" s="7" t="n"/>
+      <c r="D7" s="6" t="n"/>
       <c r="E7" s="8" t="n"/>
-      <c r="F7" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G7" s="7" t="n"/>
-    </row>
-    <row r="8">
+      <c r="F7" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
       <c r="A8" s="6" t="n"/>
       <c r="B8" s="7" t="n"/>
       <c r="C8" s="7" t="n"/>
-      <c r="D8" s="7" t="n"/>
+      <c r="D8" s="6" t="n"/>
       <c r="E8" s="8" t="n"/>
-      <c r="F8" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G8" s="7" t="n"/>
-    </row>
-    <row r="9">
+      <c r="F8" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
       <c r="A9" s="6" t="n"/>
       <c r="B9" s="7" t="n"/>
       <c r="C9" s="7" t="n"/>
-      <c r="D9" s="7" t="n"/>
+      <c r="D9" s="6" t="n"/>
       <c r="E9" s="8" t="n"/>
-      <c r="F9" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G9" s="7" t="n"/>
-    </row>
-    <row r="10">
+      <c r="F9" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
       <c r="A10" s="6" t="n"/>
       <c r="B10" s="7" t="n"/>
       <c r="C10" s="7" t="n"/>
-      <c r="D10" s="7" t="n"/>
+      <c r="D10" s="6" t="n"/>
       <c r="E10" s="8" t="n"/>
-      <c r="F10" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G10" s="7" t="n"/>
-    </row>
-    <row r="11">
+      <c r="F10" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
       <c r="A11" s="6" t="n"/>
       <c r="B11" s="7" t="n"/>
       <c r="C11" s="7" t="n"/>
-      <c r="D11" s="7" t="n"/>
+      <c r="D11" s="6" t="n"/>
       <c r="E11" s="8" t="n"/>
-      <c r="F11" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G11" s="7" t="n"/>
-    </row>
-    <row r="12">
+      <c r="F11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
       <c r="A12" s="6" t="n"/>
       <c r="B12" s="7" t="n"/>
       <c r="C12" s="7" t="n"/>
-      <c r="D12" s="7" t="n"/>
+      <c r="D12" s="6" t="n"/>
       <c r="E12" s="8" t="n"/>
-      <c r="F12" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G12" s="7" t="n"/>
-    </row>
-    <row r="13">
+      <c r="F12" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
       <c r="A13" s="6" t="n"/>
       <c r="B13" s="7" t="n"/>
       <c r="C13" s="7" t="n"/>
-      <c r="D13" s="7" t="n"/>
+      <c r="D13" s="6" t="n"/>
       <c r="E13" s="8" t="n"/>
-      <c r="F13" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G13" s="7" t="n"/>
-    </row>
-    <row r="14">
+      <c r="F13" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
       <c r="A14" s="6" t="n"/>
       <c r="B14" s="7" t="n"/>
       <c r="C14" s="7" t="n"/>
-      <c r="D14" s="7" t="n"/>
+      <c r="D14" s="6" t="n"/>
       <c r="E14" s="8" t="n"/>
-      <c r="F14" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G14" s="7" t="n"/>
-    </row>
-    <row r="15">
+      <c r="F14" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
       <c r="A15" s="6" t="n"/>
       <c r="B15" s="7" t="n"/>
       <c r="C15" s="7" t="n"/>
-      <c r="D15" s="7" t="n"/>
+      <c r="D15" s="6" t="n"/>
       <c r="E15" s="8" t="n"/>
-      <c r="F15" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G15" s="7" t="n"/>
-    </row>
-    <row r="16">
+      <c r="F15" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
       <c r="A16" s="6" t="n"/>
       <c r="B16" s="7" t="n"/>
       <c r="C16" s="7" t="n"/>
-      <c r="D16" s="7" t="n"/>
+      <c r="D16" s="6" t="n"/>
       <c r="E16" s="8" t="n"/>
-      <c r="F16" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G16" s="7" t="n"/>
-    </row>
-    <row r="17">
+      <c r="F16" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
       <c r="A17" s="6" t="n"/>
       <c r="B17" s="7" t="n"/>
       <c r="C17" s="7" t="n"/>
-      <c r="D17" s="7" t="n"/>
+      <c r="D17" s="6" t="n"/>
       <c r="E17" s="8" t="n"/>
-      <c r="F17" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G17" s="7" t="n"/>
-    </row>
-    <row r="18">
+      <c r="F17" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
       <c r="A18" s="6" t="n"/>
       <c r="B18" s="7" t="n"/>
       <c r="C18" s="7" t="n"/>
-      <c r="D18" s="7" t="n"/>
+      <c r="D18" s="6" t="n"/>
       <c r="E18" s="8" t="n"/>
-      <c r="F18" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G18" s="7" t="n"/>
-    </row>
-    <row r="19">
+      <c r="F18" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
       <c r="A19" s="6" t="n"/>
       <c r="B19" s="7" t="n"/>
       <c r="C19" s="7" t="n"/>
-      <c r="D19" s="7" t="n"/>
+      <c r="D19" s="6" t="n"/>
       <c r="E19" s="8" t="n"/>
-      <c r="F19" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G19" s="7" t="n"/>
-    </row>
-    <row r="20">
+      <c r="F19" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
       <c r="A20" s="6" t="n"/>
       <c r="B20" s="7" t="n"/>
       <c r="C20" s="7" t="n"/>
-      <c r="D20" s="7" t="n"/>
+      <c r="D20" s="6" t="n"/>
       <c r="E20" s="8" t="n"/>
-      <c r="F20" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G20" s="7" t="n"/>
-    </row>
-    <row r="21">
+      <c r="F20" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
       <c r="A21" s="6" t="n"/>
       <c r="B21" s="7" t="n"/>
       <c r="C21" s="7" t="n"/>
-      <c r="D21" s="7" t="n"/>
+      <c r="D21" s="6" t="n"/>
       <c r="E21" s="8" t="n"/>
-      <c r="F21" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G21" s="7" t="n"/>
-    </row>
-    <row r="22">
+      <c r="F21" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
       <c r="A22" s="6" t="n"/>
       <c r="B22" s="7" t="n"/>
       <c r="C22" s="7" t="n"/>
-      <c r="D22" s="7" t="n"/>
+      <c r="D22" s="6" t="n"/>
       <c r="E22" s="8" t="n"/>
-      <c r="F22" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G22" s="7" t="n"/>
-    </row>
-    <row r="23">
+      <c r="F22" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
       <c r="A23" s="6" t="n"/>
       <c r="B23" s="7" t="n"/>
       <c r="C23" s="7" t="n"/>
-      <c r="D23" s="7" t="n"/>
+      <c r="D23" s="6" t="n"/>
       <c r="E23" s="8" t="n"/>
-      <c r="F23" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G23" s="7" t="n"/>
-    </row>
-    <row r="24">
+      <c r="F23" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
       <c r="A24" s="6" t="n"/>
       <c r="B24" s="7" t="n"/>
       <c r="C24" s="7" t="n"/>
-      <c r="D24" s="7" t="n"/>
+      <c r="D24" s="6" t="n"/>
       <c r="E24" s="8" t="n"/>
-      <c r="F24" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G24" s="7" t="n"/>
-    </row>
-    <row r="25">
+      <c r="F24" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
       <c r="A25" s="6" t="n"/>
       <c r="B25" s="7" t="n"/>
       <c r="C25" s="7" t="n"/>
-      <c r="D25" s="7" t="n"/>
+      <c r="D25" s="6" t="n"/>
       <c r="E25" s="8" t="n"/>
-      <c r="F25" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G25" s="7" t="n"/>
-    </row>
-    <row r="26">
+      <c r="F25" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1">
       <c r="A26" s="6" t="n"/>
       <c r="B26" s="7" t="n"/>
       <c r="C26" s="7" t="n"/>
-      <c r="D26" s="7" t="n"/>
+      <c r="D26" s="6" t="n"/>
       <c r="E26" s="8" t="n"/>
-      <c r="F26" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G26" s="7" t="n"/>
-    </row>
-    <row r="27">
+      <c r="F26" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1">
       <c r="A27" s="6" t="n"/>
       <c r="B27" s="7" t="n"/>
       <c r="C27" s="7" t="n"/>
-      <c r="D27" s="7" t="n"/>
+      <c r="D27" s="6" t="n"/>
       <c r="E27" s="8" t="n"/>
-      <c r="F27" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G27" s="7" t="n"/>
-    </row>
-    <row r="28">
+      <c r="F27" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1">
       <c r="A28" s="6" t="n"/>
       <c r="B28" s="7" t="n"/>
       <c r="C28" s="7" t="n"/>
-      <c r="D28" s="7" t="n"/>
+      <c r="D28" s="6" t="n"/>
       <c r="E28" s="8" t="n"/>
-      <c r="F28" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G28" s="7" t="n"/>
-    </row>
-    <row r="29">
+      <c r="F28" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1">
       <c r="A29" s="6" t="n"/>
       <c r="B29" s="7" t="n"/>
       <c r="C29" s="7" t="n"/>
-      <c r="D29" s="7" t="n"/>
+      <c r="D29" s="6" t="n"/>
       <c r="E29" s="8" t="n"/>
-      <c r="F29" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G29" s="7" t="n"/>
-    </row>
-    <row r="30">
+      <c r="F29" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1">
       <c r="A30" s="6" t="n"/>
       <c r="B30" s="7" t="n"/>
       <c r="C30" s="7" t="n"/>
-      <c r="D30" s="7" t="n"/>
+      <c r="D30" s="6" t="n"/>
       <c r="E30" s="8" t="n"/>
-      <c r="F30" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G30" s="7" t="n"/>
-    </row>
-    <row r="31">
+      <c r="F30" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1">
       <c r="A31" s="6" t="n"/>
       <c r="B31" s="7" t="n"/>
       <c r="C31" s="7" t="n"/>
-      <c r="D31" s="7" t="n"/>
+      <c r="D31" s="6" t="n"/>
       <c r="E31" s="8" t="n"/>
-      <c r="F31" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G31" s="7" t="n"/>
-    </row>
-    <row r="32">
+      <c r="F31" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G31" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1">
       <c r="A32" s="6" t="n"/>
       <c r="B32" s="7" t="n"/>
       <c r="C32" s="7" t="n"/>
-      <c r="D32" s="7" t="n"/>
+      <c r="D32" s="6" t="n"/>
       <c r="E32" s="8" t="n"/>
-      <c r="F32" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G32" s="7" t="n"/>
-    </row>
-    <row r="33">
+      <c r="F32" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1">
       <c r="A33" s="6" t="n"/>
       <c r="B33" s="7" t="n"/>
       <c r="C33" s="7" t="n"/>
-      <c r="D33" s="7" t="n"/>
+      <c r="D33" s="6" t="n"/>
       <c r="E33" s="8" t="n"/>
-      <c r="F33" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G33" s="7" t="n"/>
-    </row>
-    <row r="34">
+      <c r="F33" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G33" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="18" customHeight="1">
       <c r="A34" s="6" t="n"/>
       <c r="B34" s="7" t="n"/>
       <c r="C34" s="7" t="n"/>
-      <c r="D34" s="7" t="n"/>
+      <c r="D34" s="6" t="n"/>
       <c r="E34" s="8" t="n"/>
-      <c r="F34" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G34" s="7" t="n"/>
-    </row>
-    <row r="35">
+      <c r="F34" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G34" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="18" customHeight="1">
       <c r="A35" s="6" t="n"/>
       <c r="B35" s="7" t="n"/>
       <c r="C35" s="7" t="n"/>
-      <c r="D35" s="7" t="n"/>
+      <c r="D35" s="6" t="n"/>
       <c r="E35" s="8" t="n"/>
-      <c r="F35" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G35" s="7" t="n"/>
-    </row>
-    <row r="36">
+      <c r="F35" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G35" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1">
       <c r="A36" s="6" t="n"/>
       <c r="B36" s="7" t="n"/>
       <c r="C36" s="7" t="n"/>
-      <c r="D36" s="7" t="n"/>
+      <c r="D36" s="6" t="n"/>
       <c r="E36" s="8" t="n"/>
-      <c r="F36" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G36" s="7" t="n"/>
-    </row>
-    <row r="37">
+      <c r="F36" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G36" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="18" customHeight="1">
       <c r="A37" s="6" t="n"/>
       <c r="B37" s="7" t="n"/>
       <c r="C37" s="7" t="n"/>
-      <c r="D37" s="7" t="n"/>
+      <c r="D37" s="6" t="n"/>
       <c r="E37" s="8" t="n"/>
-      <c r="F37" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G37" s="7" t="n"/>
-    </row>
-    <row r="38">
+      <c r="F37" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G37" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="18" customHeight="1">
       <c r="A38" s="6" t="n"/>
       <c r="B38" s="7" t="n"/>
       <c r="C38" s="7" t="n"/>
-      <c r="D38" s="7" t="n"/>
+      <c r="D38" s="6" t="n"/>
       <c r="E38" s="8" t="n"/>
-      <c r="F38" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G38" s="7" t="n"/>
-    </row>
-    <row r="39">
+      <c r="F38" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G38" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="18" customHeight="1">
       <c r="A39" s="6" t="n"/>
       <c r="B39" s="7" t="n"/>
       <c r="C39" s="7" t="n"/>
-      <c r="D39" s="7" t="n"/>
+      <c r="D39" s="6" t="n"/>
       <c r="E39" s="8" t="n"/>
-      <c r="F39" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G39" s="7" t="n"/>
-    </row>
-    <row r="40">
+      <c r="F39" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G39" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1">
       <c r="A40" s="6" t="n"/>
       <c r="B40" s="7" t="n"/>
       <c r="C40" s="7" t="n"/>
-      <c r="D40" s="7" t="n"/>
+      <c r="D40" s="6" t="n"/>
       <c r="E40" s="8" t="n"/>
-      <c r="F40" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G40" s="7" t="n"/>
-    </row>
-    <row r="41">
+      <c r="F40" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G40" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="18" customHeight="1">
       <c r="A41" s="6" t="n"/>
       <c r="B41" s="7" t="n"/>
       <c r="C41" s="7" t="n"/>
-      <c r="D41" s="7" t="n"/>
+      <c r="D41" s="6" t="n"/>
       <c r="E41" s="8" t="n"/>
-      <c r="F41" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G41" s="7" t="n"/>
-    </row>
-    <row r="42">
+      <c r="F41" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G41" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="18" customHeight="1">
       <c r="A42" s="6" t="n"/>
       <c r="B42" s="7" t="n"/>
       <c r="C42" s="7" t="n"/>
-      <c r="D42" s="7" t="n"/>
+      <c r="D42" s="6" t="n"/>
       <c r="E42" s="8" t="n"/>
-      <c r="F42" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G42" s="7" t="n"/>
-    </row>
-    <row r="43">
+      <c r="F42" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="18" customHeight="1">
       <c r="A43" s="6" t="n"/>
       <c r="B43" s="7" t="n"/>
       <c r="C43" s="7" t="n"/>
-      <c r="D43" s="7" t="n"/>
+      <c r="D43" s="6" t="n"/>
       <c r="E43" s="8" t="n"/>
-      <c r="F43" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G43" s="7" t="n"/>
-    </row>
-    <row r="44">
+      <c r="F43" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G43" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="18" customHeight="1">
       <c r="A44" s="6" t="n"/>
       <c r="B44" s="7" t="n"/>
       <c r="C44" s="7" t="n"/>
-      <c r="D44" s="7" t="n"/>
+      <c r="D44" s="6" t="n"/>
       <c r="E44" s="8" t="n"/>
-      <c r="F44" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G44" s="7" t="n"/>
-    </row>
-    <row r="45">
+      <c r="F44" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G44" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="18" customHeight="1">
       <c r="A45" s="6" t="n"/>
       <c r="B45" s="7" t="n"/>
       <c r="C45" s="7" t="n"/>
-      <c r="D45" s="7" t="n"/>
+      <c r="D45" s="6" t="n"/>
       <c r="E45" s="8" t="n"/>
-      <c r="F45" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G45" s="7" t="n"/>
-    </row>
-    <row r="46">
+      <c r="F45" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G45" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="18" customHeight="1">
       <c r="A46" s="6" t="n"/>
       <c r="B46" s="7" t="n"/>
       <c r="C46" s="7" t="n"/>
-      <c r="D46" s="7" t="n"/>
+      <c r="D46" s="6" t="n"/>
       <c r="E46" s="8" t="n"/>
-      <c r="F46" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G46" s="7" t="n"/>
-    </row>
-    <row r="47">
+      <c r="F46" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G46" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="18" customHeight="1">
       <c r="A47" s="6" t="n"/>
       <c r="B47" s="7" t="n"/>
       <c r="C47" s="7" t="n"/>
-      <c r="D47" s="7" t="n"/>
+      <c r="D47" s="6" t="n"/>
       <c r="E47" s="8" t="n"/>
-      <c r="F47" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G47" s="7" t="n"/>
-    </row>
-    <row r="48">
+      <c r="F47" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G47" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="18" customHeight="1">
       <c r="A48" s="6" t="n"/>
       <c r="B48" s="7" t="n"/>
       <c r="C48" s="7" t="n"/>
-      <c r="D48" s="7" t="n"/>
+      <c r="D48" s="6" t="n"/>
       <c r="E48" s="8" t="n"/>
-      <c r="F48" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G48" s="7" t="n"/>
-    </row>
-    <row r="49">
+      <c r="F48" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G48" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="18" customHeight="1">
       <c r="A49" s="6" t="n"/>
       <c r="B49" s="7" t="n"/>
       <c r="C49" s="7" t="n"/>
-      <c r="D49" s="7" t="n"/>
+      <c r="D49" s="6" t="n"/>
       <c r="E49" s="8" t="n"/>
-      <c r="F49" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G49" s="7" t="n"/>
-    </row>
-    <row r="50">
+      <c r="F49" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G49" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="18" customHeight="1">
       <c r="A50" s="6" t="n"/>
       <c r="B50" s="7" t="n"/>
       <c r="C50" s="7" t="n"/>
-      <c r="D50" s="7" t="n"/>
+      <c r="D50" s="6" t="n"/>
       <c r="E50" s="8" t="n"/>
-      <c r="F50" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G50" s="7" t="n"/>
-    </row>
-    <row r="51">
+      <c r="F50" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G50" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="18" customHeight="1">
       <c r="A51" s="6" t="n"/>
       <c r="B51" s="7" t="n"/>
       <c r="C51" s="7" t="n"/>
-      <c r="D51" s="7" t="n"/>
+      <c r="D51" s="6" t="n"/>
       <c r="E51" s="8" t="n"/>
-      <c r="F51" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G51" s="7" t="n"/>
-    </row>
-    <row r="52">
+      <c r="F51" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G51" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="18" customHeight="1">
       <c r="A52" s="6" t="n"/>
       <c r="B52" s="7" t="n"/>
       <c r="C52" s="7" t="n"/>
-      <c r="D52" s="7" t="n"/>
+      <c r="D52" s="6" t="n"/>
       <c r="E52" s="8" t="n"/>
-      <c r="F52" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G52" s="7" t="n"/>
-    </row>
-    <row r="53">
+      <c r="F52" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G52" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="18" customHeight="1">
       <c r="A53" s="6" t="n"/>
       <c r="B53" s="7" t="n"/>
       <c r="C53" s="7" t="n"/>
-      <c r="D53" s="7" t="n"/>
+      <c r="D53" s="6" t="n"/>
       <c r="E53" s="8" t="n"/>
-      <c r="F53" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G53" s="7" t="n"/>
-    </row>
-    <row r="54">
+      <c r="F53" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G53" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="18" customHeight="1">
       <c r="A54" s="6" t="n"/>
       <c r="B54" s="7" t="n"/>
       <c r="C54" s="7" t="n"/>
-      <c r="D54" s="7" t="n"/>
+      <c r="D54" s="6" t="n"/>
       <c r="E54" s="8" t="n"/>
-      <c r="F54" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G54" s="7" t="n"/>
-    </row>
-    <row r="55">
+      <c r="F54" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G54" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="18" customHeight="1">
       <c r="A55" s="6" t="n"/>
       <c r="B55" s="7" t="n"/>
       <c r="C55" s="7" t="n"/>
-      <c r="D55" s="7" t="n"/>
+      <c r="D55" s="6" t="n"/>
       <c r="E55" s="8" t="n"/>
-      <c r="F55" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G55" s="7" t="n"/>
-    </row>
-    <row r="56">
+      <c r="F55" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G55" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="18" customHeight="1">
       <c r="A56" s="6" t="n"/>
       <c r="B56" s="7" t="n"/>
       <c r="C56" s="7" t="n"/>
-      <c r="D56" s="7" t="n"/>
+      <c r="D56" s="6" t="n"/>
       <c r="E56" s="8" t="n"/>
-      <c r="F56" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G56" s="7" t="n"/>
-    </row>
-    <row r="57">
+      <c r="F56" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G56" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="18" customHeight="1">
       <c r="A57" s="6" t="n"/>
       <c r="B57" s="7" t="n"/>
       <c r="C57" s="7" t="n"/>
-      <c r="D57" s="7" t="n"/>
+      <c r="D57" s="6" t="n"/>
       <c r="E57" s="8" t="n"/>
-      <c r="F57" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G57" s="7" t="n"/>
-    </row>
-    <row r="58">
+      <c r="F57" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G57" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="18" customHeight="1">
       <c r="A58" s="6" t="n"/>
       <c r="B58" s="7" t="n"/>
       <c r="C58" s="7" t="n"/>
-      <c r="D58" s="7" t="n"/>
+      <c r="D58" s="6" t="n"/>
       <c r="E58" s="8" t="n"/>
-      <c r="F58" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G58" s="7" t="n"/>
-    </row>
-    <row r="59">
+      <c r="F58" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G58" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="18" customHeight="1">
       <c r="A59" s="6" t="n"/>
       <c r="B59" s="7" t="n"/>
       <c r="C59" s="7" t="n"/>
-      <c r="D59" s="7" t="n"/>
+      <c r="D59" s="6" t="n"/>
       <c r="E59" s="8" t="n"/>
-      <c r="F59" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G59" s="7" t="n"/>
-    </row>
-    <row r="60">
+      <c r="F59" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G59" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="18" customHeight="1">
       <c r="A60" s="6" t="n"/>
       <c r="B60" s="7" t="n"/>
       <c r="C60" s="7" t="n"/>
-      <c r="D60" s="7" t="n"/>
+      <c r="D60" s="6" t="n"/>
       <c r="E60" s="8" t="n"/>
-      <c r="F60" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G60" s="7" t="n"/>
-    </row>
-    <row r="61">
+      <c r="F60" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G60" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="18" customHeight="1">
       <c r="A61" s="6" t="n"/>
       <c r="B61" s="7" t="n"/>
       <c r="C61" s="7" t="n"/>
-      <c r="D61" s="7" t="n"/>
+      <c r="D61" s="6" t="n"/>
       <c r="E61" s="8" t="n"/>
-      <c r="F61" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G61" s="7" t="n"/>
-    </row>
-    <row r="62">
+      <c r="F61" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G61" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="18" customHeight="1">
       <c r="A62" s="6" t="n"/>
       <c r="B62" s="7" t="n"/>
       <c r="C62" s="7" t="n"/>
-      <c r="D62" s="7" t="n"/>
+      <c r="D62" s="6" t="n"/>
       <c r="E62" s="8" t="n"/>
-      <c r="F62" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G62" s="7" t="n"/>
-    </row>
-    <row r="63">
+      <c r="F62" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G62" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="18" customHeight="1">
       <c r="A63" s="6" t="n"/>
       <c r="B63" s="7" t="n"/>
       <c r="C63" s="7" t="n"/>
-      <c r="D63" s="7" t="n"/>
+      <c r="D63" s="6" t="n"/>
       <c r="E63" s="8" t="n"/>
-      <c r="F63" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G63" s="7" t="n"/>
-    </row>
-    <row r="64">
+      <c r="F63" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G63" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="18" customHeight="1">
       <c r="A64" s="6" t="n"/>
       <c r="B64" s="7" t="n"/>
       <c r="C64" s="7" t="n"/>
-      <c r="D64" s="7" t="n"/>
+      <c r="D64" s="6" t="n"/>
       <c r="E64" s="8" t="n"/>
-      <c r="F64" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G64" s="7" t="n"/>
-    </row>
-    <row r="65">
+      <c r="F64" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G64" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="18" customHeight="1">
       <c r="A65" s="6" t="n"/>
       <c r="B65" s="7" t="n"/>
       <c r="C65" s="7" t="n"/>
-      <c r="D65" s="7" t="n"/>
+      <c r="D65" s="6" t="n"/>
       <c r="E65" s="8" t="n"/>
-      <c r="F65" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G65" s="7" t="n"/>
-    </row>
-    <row r="66">
+      <c r="F65" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G65" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="18" customHeight="1">
       <c r="A66" s="6" t="n"/>
       <c r="B66" s="7" t="n"/>
       <c r="C66" s="7" t="n"/>
-      <c r="D66" s="7" t="n"/>
+      <c r="D66" s="6" t="n"/>
       <c r="E66" s="8" t="n"/>
-      <c r="F66" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G66" s="7" t="n"/>
-    </row>
-    <row r="67">
+      <c r="F66" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G66" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="18" customHeight="1">
       <c r="A67" s="6" t="n"/>
       <c r="B67" s="7" t="n"/>
       <c r="C67" s="7" t="n"/>
-      <c r="D67" s="7" t="n"/>
+      <c r="D67" s="6" t="n"/>
       <c r="E67" s="8" t="n"/>
-      <c r="F67" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G67" s="7" t="n"/>
-    </row>
-    <row r="68">
+      <c r="F67" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G67" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="18" customHeight="1">
       <c r="A68" s="6" t="n"/>
       <c r="B68" s="7" t="n"/>
       <c r="C68" s="7" t="n"/>
-      <c r="D68" s="7" t="n"/>
+      <c r="D68" s="6" t="n"/>
       <c r="E68" s="8" t="n"/>
-      <c r="F68" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G68" s="7" t="n"/>
-    </row>
-    <row r="69">
+      <c r="F68" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G68" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="18" customHeight="1">
       <c r="A69" s="6" t="n"/>
       <c r="B69" s="7" t="n"/>
       <c r="C69" s="7" t="n"/>
-      <c r="D69" s="7" t="n"/>
+      <c r="D69" s="6" t="n"/>
       <c r="E69" s="8" t="n"/>
-      <c r="F69" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G69" s="7" t="n"/>
-    </row>
-    <row r="70">
+      <c r="F69" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G69" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="18" customHeight="1">
       <c r="A70" s="6" t="n"/>
       <c r="B70" s="7" t="n"/>
       <c r="C70" s="7" t="n"/>
-      <c r="D70" s="7" t="n"/>
+      <c r="D70" s="6" t="n"/>
       <c r="E70" s="8" t="n"/>
-      <c r="F70" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G70" s="7" t="n"/>
-    </row>
-    <row r="71">
+      <c r="F70" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G70" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="18" customHeight="1">
       <c r="A71" s="6" t="n"/>
       <c r="B71" s="7" t="n"/>
       <c r="C71" s="7" t="n"/>
-      <c r="D71" s="7" t="n"/>
+      <c r="D71" s="6" t="n"/>
       <c r="E71" s="8" t="n"/>
-      <c r="F71" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G71" s="7" t="n"/>
-    </row>
-    <row r="72">
+      <c r="F71" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G71" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="18" customHeight="1">
       <c r="A72" s="6" t="n"/>
       <c r="B72" s="7" t="n"/>
       <c r="C72" s="7" t="n"/>
-      <c r="D72" s="7" t="n"/>
+      <c r="D72" s="6" t="n"/>
       <c r="E72" s="8" t="n"/>
-      <c r="F72" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G72" s="7" t="n"/>
-    </row>
-    <row r="73">
+      <c r="F72" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G72" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="18" customHeight="1">
       <c r="A73" s="6" t="n"/>
       <c r="B73" s="7" t="n"/>
       <c r="C73" s="7" t="n"/>
-      <c r="D73" s="7" t="n"/>
+      <c r="D73" s="6" t="n"/>
       <c r="E73" s="8" t="n"/>
-      <c r="F73" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G73" s="7" t="n"/>
-    </row>
-    <row r="74">
+      <c r="F73" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G73" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="18" customHeight="1">
       <c r="A74" s="6" t="n"/>
       <c r="B74" s="7" t="n"/>
       <c r="C74" s="7" t="n"/>
-      <c r="D74" s="7" t="n"/>
+      <c r="D74" s="6" t="n"/>
       <c r="E74" s="8" t="n"/>
-      <c r="F74" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G74" s="7" t="n"/>
-    </row>
-    <row r="75">
+      <c r="F74" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G74" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="18" customHeight="1">
       <c r="A75" s="6" t="n"/>
       <c r="B75" s="7" t="n"/>
       <c r="C75" s="7" t="n"/>
-      <c r="D75" s="7" t="n"/>
+      <c r="D75" s="6" t="n"/>
       <c r="E75" s="8" t="n"/>
-      <c r="F75" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G75" s="7" t="n"/>
-    </row>
-    <row r="76">
+      <c r="F75" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G75" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="18" customHeight="1">
       <c r="A76" s="6" t="n"/>
       <c r="B76" s="7" t="n"/>
       <c r="C76" s="7" t="n"/>
-      <c r="D76" s="7" t="n"/>
+      <c r="D76" s="6" t="n"/>
       <c r="E76" s="8" t="n"/>
-      <c r="F76" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G76" s="7" t="n"/>
-    </row>
-    <row r="77">
+      <c r="F76" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G76" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="18" customHeight="1">
       <c r="A77" s="6" t="n"/>
       <c r="B77" s="7" t="n"/>
       <c r="C77" s="7" t="n"/>
-      <c r="D77" s="7" t="n"/>
+      <c r="D77" s="6" t="n"/>
       <c r="E77" s="8" t="n"/>
-      <c r="F77" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G77" s="7" t="n"/>
-    </row>
-    <row r="78">
+      <c r="F77" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G77" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="18" customHeight="1">
       <c r="A78" s="6" t="n"/>
       <c r="B78" s="7" t="n"/>
       <c r="C78" s="7" t="n"/>
-      <c r="D78" s="7" t="n"/>
+      <c r="D78" s="6" t="n"/>
       <c r="E78" s="8" t="n"/>
-      <c r="F78" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G78" s="7" t="n"/>
-    </row>
-    <row r="79">
+      <c r="F78" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G78" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="18" customHeight="1">
       <c r="A79" s="6" t="n"/>
       <c r="B79" s="7" t="n"/>
       <c r="C79" s="7" t="n"/>
-      <c r="D79" s="7" t="n"/>
+      <c r="D79" s="6" t="n"/>
       <c r="E79" s="8" t="n"/>
-      <c r="F79" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G79" s="7" t="n"/>
-    </row>
-    <row r="80">
+      <c r="F79" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G79" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="18" customHeight="1">
       <c r="A80" s="6" t="n"/>
       <c r="B80" s="7" t="n"/>
       <c r="C80" s="7" t="n"/>
-      <c r="D80" s="7" t="n"/>
+      <c r="D80" s="6" t="n"/>
       <c r="E80" s="8" t="n"/>
-      <c r="F80" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G80" s="7" t="n"/>
-    </row>
-    <row r="81">
+      <c r="F80" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G80" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="18" customHeight="1">
       <c r="A81" s="6" t="n"/>
       <c r="B81" s="7" t="n"/>
       <c r="C81" s="7" t="n"/>
-      <c r="D81" s="7" t="n"/>
+      <c r="D81" s="6" t="n"/>
       <c r="E81" s="8" t="n"/>
-      <c r="F81" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G81" s="7" t="n"/>
-    </row>
-    <row r="82">
+      <c r="F81" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G81" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="18" customHeight="1">
       <c r="A82" s="6" t="n"/>
       <c r="B82" s="7" t="n"/>
       <c r="C82" s="7" t="n"/>
-      <c r="D82" s="7" t="n"/>
+      <c r="D82" s="6" t="n"/>
       <c r="E82" s="8" t="n"/>
-      <c r="F82" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G82" s="7" t="n"/>
-    </row>
-    <row r="83">
+      <c r="F82" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G82" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="18" customHeight="1">
       <c r="A83" s="6" t="n"/>
       <c r="B83" s="7" t="n"/>
       <c r="C83" s="7" t="n"/>
-      <c r="D83" s="7" t="n"/>
+      <c r="D83" s="6" t="n"/>
       <c r="E83" s="8" t="n"/>
-      <c r="F83" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G83" s="7" t="n"/>
-    </row>
-    <row r="84">
+      <c r="F83" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G83" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="18" customHeight="1">
       <c r="A84" s="6" t="n"/>
       <c r="B84" s="7" t="n"/>
       <c r="C84" s="7" t="n"/>
-      <c r="D84" s="7" t="n"/>
+      <c r="D84" s="6" t="n"/>
       <c r="E84" s="8" t="n"/>
-      <c r="F84" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G84" s="7" t="n"/>
-    </row>
-    <row r="85">
+      <c r="F84" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G84" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="18" customHeight="1">
       <c r="A85" s="6" t="n"/>
       <c r="B85" s="7" t="n"/>
       <c r="C85" s="7" t="n"/>
-      <c r="D85" s="7" t="n"/>
+      <c r="D85" s="6" t="n"/>
       <c r="E85" s="8" t="n"/>
-      <c r="F85" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G85" s="7" t="n"/>
-    </row>
-    <row r="86">
+      <c r="F85" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G85" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="18" customHeight="1">
       <c r="A86" s="6" t="n"/>
       <c r="B86" s="7" t="n"/>
       <c r="C86" s="7" t="n"/>
-      <c r="D86" s="7" t="n"/>
+      <c r="D86" s="6" t="n"/>
       <c r="E86" s="8" t="n"/>
-      <c r="F86" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G86" s="7" t="n"/>
-    </row>
-    <row r="87">
+      <c r="F86" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G86" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="18" customHeight="1">
       <c r="A87" s="6" t="n"/>
       <c r="B87" s="7" t="n"/>
       <c r="C87" s="7" t="n"/>
-      <c r="D87" s="7" t="n"/>
+      <c r="D87" s="6" t="n"/>
       <c r="E87" s="8" t="n"/>
-      <c r="F87" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G87" s="7" t="n"/>
-    </row>
-    <row r="88">
+      <c r="F87" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G87" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="18" customHeight="1">
       <c r="A88" s="6" t="n"/>
       <c r="B88" s="7" t="n"/>
       <c r="C88" s="7" t="n"/>
-      <c r="D88" s="7" t="n"/>
+      <c r="D88" s="6" t="n"/>
       <c r="E88" s="8" t="n"/>
-      <c r="F88" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G88" s="7" t="n"/>
-    </row>
-    <row r="89">
+      <c r="F88" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G88" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="18" customHeight="1">
       <c r="A89" s="6" t="n"/>
       <c r="B89" s="7" t="n"/>
       <c r="C89" s="7" t="n"/>
-      <c r="D89" s="7" t="n"/>
+      <c r="D89" s="6" t="n"/>
       <c r="E89" s="8" t="n"/>
-      <c r="F89" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G89" s="7" t="n"/>
-    </row>
-    <row r="90">
+      <c r="F89" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G89" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="18" customHeight="1">
       <c r="A90" s="6" t="n"/>
       <c r="B90" s="7" t="n"/>
       <c r="C90" s="7" t="n"/>
-      <c r="D90" s="7" t="n"/>
+      <c r="D90" s="6" t="n"/>
       <c r="E90" s="8" t="n"/>
-      <c r="F90" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G90" s="7" t="n"/>
-    </row>
-    <row r="91">
+      <c r="F90" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G90" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="18" customHeight="1">
       <c r="A91" s="6" t="n"/>
       <c r="B91" s="7" t="n"/>
       <c r="C91" s="7" t="n"/>
-      <c r="D91" s="7" t="n"/>
+      <c r="D91" s="6" t="n"/>
       <c r="E91" s="8" t="n"/>
-      <c r="F91" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G91" s="7" t="n"/>
-    </row>
-    <row r="92">
+      <c r="F91" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G91" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="18" customHeight="1">
       <c r="A92" s="6" t="n"/>
       <c r="B92" s="7" t="n"/>
       <c r="C92" s="7" t="n"/>
-      <c r="D92" s="7" t="n"/>
+      <c r="D92" s="6" t="n"/>
       <c r="E92" s="8" t="n"/>
-      <c r="F92" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G92" s="7" t="n"/>
-    </row>
-    <row r="93">
+      <c r="F92" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G92" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="18" customHeight="1">
       <c r="A93" s="6" t="n"/>
       <c r="B93" s="7" t="n"/>
       <c r="C93" s="7" t="n"/>
-      <c r="D93" s="7" t="n"/>
+      <c r="D93" s="6" t="n"/>
       <c r="E93" s="8" t="n"/>
-      <c r="F93" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G93" s="7" t="n"/>
-    </row>
-    <row r="94">
+      <c r="F93" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G93" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="18" customHeight="1">
       <c r="A94" s="6" t="n"/>
       <c r="B94" s="7" t="n"/>
       <c r="C94" s="7" t="n"/>
-      <c r="D94" s="7" t="n"/>
+      <c r="D94" s="6" t="n"/>
       <c r="E94" s="8" t="n"/>
-      <c r="F94" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G94" s="7" t="n"/>
-    </row>
-    <row r="95">
+      <c r="F94" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G94" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="18" customHeight="1">
       <c r="A95" s="6" t="n"/>
       <c r="B95" s="7" t="n"/>
       <c r="C95" s="7" t="n"/>
-      <c r="D95" s="7" t="n"/>
+      <c r="D95" s="6" t="n"/>
       <c r="E95" s="8" t="n"/>
-      <c r="F95" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G95" s="7" t="n"/>
-    </row>
-    <row r="96">
+      <c r="F95" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G95" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="18" customHeight="1">
       <c r="A96" s="6" t="n"/>
       <c r="B96" s="7" t="n"/>
       <c r="C96" s="7" t="n"/>
-      <c r="D96" s="7" t="n"/>
+      <c r="D96" s="6" t="n"/>
       <c r="E96" s="8" t="n"/>
-      <c r="F96" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G96" s="7" t="n"/>
-    </row>
-    <row r="97">
+      <c r="F96" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G96" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="18" customHeight="1">
       <c r="A97" s="6" t="n"/>
       <c r="B97" s="7" t="n"/>
       <c r="C97" s="7" t="n"/>
-      <c r="D97" s="7" t="n"/>
+      <c r="D97" s="6" t="n"/>
       <c r="E97" s="8" t="n"/>
-      <c r="F97" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G97" s="7" t="n"/>
-    </row>
-    <row r="98">
+      <c r="F97" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G97" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="18" customHeight="1">
       <c r="A98" s="6" t="n"/>
       <c r="B98" s="7" t="n"/>
       <c r="C98" s="7" t="n"/>
-      <c r="D98" s="7" t="n"/>
+      <c r="D98" s="6" t="n"/>
       <c r="E98" s="8" t="n"/>
-      <c r="F98" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G98" s="7" t="n"/>
-    </row>
-    <row r="99">
+      <c r="F98" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G98" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="18" customHeight="1">
       <c r="A99" s="6" t="n"/>
       <c r="B99" s="7" t="n"/>
       <c r="C99" s="7" t="n"/>
-      <c r="D99" s="7" t="n"/>
+      <c r="D99" s="6" t="n"/>
       <c r="E99" s="8" t="n"/>
-      <c r="F99" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G99" s="7" t="n"/>
-    </row>
-    <row r="100">
+      <c r="F99" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G99" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="18" customHeight="1">
       <c r="A100" s="6" t="n"/>
       <c r="B100" s="7" t="n"/>
       <c r="C100" s="7" t="n"/>
-      <c r="D100" s="7" t="n"/>
+      <c r="D100" s="6" t="n"/>
       <c r="E100" s="8" t="n"/>
-      <c r="F100" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G100" s="7" t="n"/>
-    </row>
-    <row r="101">
+      <c r="F100" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G100" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="18" customHeight="1">
       <c r="A101" s="6" t="n"/>
       <c r="B101" s="7" t="n"/>
       <c r="C101" s="7" t="n"/>
-      <c r="D101" s="7" t="n"/>
+      <c r="D101" s="6" t="n"/>
       <c r="E101" s="8" t="n"/>
-      <c r="F101" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G101" s="7" t="n"/>
-    </row>
-    <row r="102">
+      <c r="F101" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G101" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="18" customHeight="1">
       <c r="A102" s="6" t="n"/>
       <c r="B102" s="7" t="n"/>
       <c r="C102" s="7" t="n"/>
-      <c r="D102" s="7" t="n"/>
+      <c r="D102" s="6" t="n"/>
       <c r="E102" s="8" t="n"/>
-      <c r="F102" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G102" s="7" t="n"/>
-    </row>
-    <row r="103">
+      <c r="F102" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G102" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="18" customHeight="1">
       <c r="A103" s="6" t="n"/>
       <c r="B103" s="7" t="n"/>
       <c r="C103" s="7" t="n"/>
-      <c r="D103" s="7" t="n"/>
+      <c r="D103" s="6" t="n"/>
       <c r="E103" s="8" t="n"/>
-      <c r="F103" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G103" s="7" t="n"/>
-    </row>
-    <row r="104">
+      <c r="F103" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G103" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="18" customHeight="1">
       <c r="A104" s="6" t="n"/>
       <c r="B104" s="7" t="n"/>
       <c r="C104" s="7" t="n"/>
-      <c r="D104" s="7" t="n"/>
+      <c r="D104" s="6" t="n"/>
       <c r="E104" s="8" t="n"/>
-      <c r="F104" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="G104" s="7" t="n"/>
+      <c r="F104" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="G104" s="6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
-  <dataValidations count="2">
-    <dataValidation sqref="G5:G104" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor inválido" error="Digite SIM ou NÃO" type="list">
+  <dataValidations count="3">
+    <dataValidation sqref="G5:G104" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Valor inválido" error="Digite SIM ou NÃO" type="list">
       <formula1>"SIM,NÃO"</formula1>
     </dataValidation>
-    <dataValidation sqref="F5:F104" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Horas inválidas" error="Digite entre 1 e 24" type="decimal" operator="between">
+    <dataValidation sqref="F5:F104" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Horas inválidas" error="Digite entre 1 e 24" type="decimal" operator="between">
       <formula1>1</formula1>
       <formula2>24</formula2>
+    </dataValidation>
+    <dataValidation sqref="E5:E104" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Custo inválido" error="Digite um valor &gt;= 0" type="decimal" operator="greaterThanOrEqual">
+      <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1815,7 +2228,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -2067,168 +2480,161 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A25"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="80" customWidth="1" min="1" max="1"/>
+    <col width="85" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="26" customHeight="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" s="15" t="inlineStr">
         <is>
           <t>INSTRUÇÕES DE PREENCHIMENTO</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="8" customHeight="1">
+    <row r="2" ht="6" customHeight="1">
       <c r="A2" s="16" t="inlineStr"/>
     </row>
-    <row r="3" ht="20" customHeight="1">
+    <row r="3" ht="22" customHeight="1">
       <c r="A3" s="17" t="inlineStr">
         <is>
-          <t>1. CAMPOS OBRIGATÓRIOS (fundo rosa)</t>
+          <t>CAMPOS OBRIGATÓRIOS (fundo rosa)</t>
         </is>
       </c>
     </row>
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">   • Nome Completo: Informe o nome completo do funcionário.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="8" customHeight="1">
-      <c r="A5" s="16" t="inlineStr"/>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="19" t="inlineStr">
-        <is>
-          <t>2. CAMPOS OPCIONAIS (fundo azul claro)</t>
+          <t xml:space="preserve">  • Nome Completo: Nome completo do funcionário.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Cargo / Função: Função que o funcionário exerce na empresa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Custo por Hora (R$): Valor em reais por hora trabalhada.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">   • E-mail: E-mail profissional do funcionário.</t>
+          <t xml:space="preserve">  • Horas por Dia Útil: Padrão = 9h. Aceita valores entre 1 e 24.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1">
       <c r="A8" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">   • Telefone: Formato sugerido: (37) 99999-9999</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   • Cargo / Função: Consulte a aba 'Cargos de Referência' para sugestões.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   • Custo por Hora: Valor em R$ (use ponto ou vírgula como decimal).</t>
+          <t xml:space="preserve">  • Ativo (SIM/NÃO): SIM = funcionário ativo, NÃO = inativo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="6" customHeight="1">
+      <c r="A9" s="16" t="inlineStr"/>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>CAMPOS OPCIONAIS (fundo azul)</t>
         </is>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">   • Horas por Dia Útil: Padrão = 9 horas. Aceita valores entre 1 e 24.</t>
+          <t xml:space="preserve">  • E-mail: E-mail profissional do funcionário.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">   • Ativo: Digite SIM (funcionário ativo) ou NÃO (inativo). Padrão = SIM.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="8" customHeight="1">
+          <t xml:space="preserve">  • Telefone: Formato sugerido: (37) 99999-9999</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="6" customHeight="1">
       <c r="A13" s="16" t="inlineStr"/>
     </row>
-    <row r="14" ht="20" customHeight="1">
+    <row r="14" ht="22" customHeight="1">
       <c r="A14" s="20" t="inlineStr">
         <is>
-          <t>3. COMO IMPORTAR</t>
+          <t>COMO IMPORTAR</t>
         </is>
       </c>
     </row>
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">   1. Preencha os dados a partir da linha 5 (não altere as linhas 1-4).</t>
+          <t xml:space="preserve">  1. Preencha os dados a partir da linha 5 (não altere as linhas 1–4).</t>
         </is>
       </c>
     </row>
     <row r="16" ht="16" customHeight="1">
       <c r="A16" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">   2. Salve o arquivo no formato .xlsx</t>
+          <t xml:space="preserve">  2. Salve no formato .xlsx</t>
         </is>
       </c>
     </row>
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">   3. No sistema BCM, vá em Funcionários → botão 'Importar Excel'.</t>
+          <t xml:space="preserve">  3. No sistema → Funcionários → botão 'Importar Excel'.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="16" customHeight="1">
       <c r="A18" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">   4. Selecione este arquivo e confirme a importação.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   5. O sistema validará os dados e importará todos os funcionários.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="8" customHeight="1">
-      <c r="A20" s="16" t="inlineStr"/>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="21" t="inlineStr">
-        <is>
-          <t>4. DICAS</t>
+          <t xml:space="preserve">  4. Revise a pré-visualização e confirme a importação.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="6" customHeight="1">
+      <c r="A19" s="16" t="inlineStr"/>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="21" t="inlineStr">
+        <is>
+          <t>OBSERVAÇÕES</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="16" customHeight="1">
+      <c r="A21" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Não altere os cabeçalhos (linha 3) nem a estrutura das colunas.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
       <c r="A22" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">   • Não altere os cabeçalhos (linha 3) nem a estrutura das colunas.</t>
+          <t xml:space="preserve">  • A linha verde (linha 4) é apenas exemplo — não será importada.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="16" customHeight="1">
       <c r="A23" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">   • A linha verde (linha 4) é apenas um exemplo — não será importada.</t>
+          <t xml:space="preserve">  • Máximo de 100 funcionários por importação.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="16" customHeight="1">
       <c r="A24" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">   • Você pode importar até 100 funcionários por vez.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="16" customHeight="1">
-      <c r="A25" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   • Funcionários já cadastrados com o mesmo e-mail serão ignorados.</t>
+          <t xml:space="preserve">  • Consulte a aba 'Cargos de Referência' para sugestões de função.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: setor de trabalho + custos por setor + template atualizado
</commit_message>
<xml_diff>
--- a/docs/template_funcionarios.xlsx
+++ b/docs/template_funcionarios.xlsx
@@ -8,8 +8,8 @@
   </bookViews>
   <sheets>
     <sheet name="Funcionários" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Cargos de Referência" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Instruções" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Setores de Trabalho" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Cargos de Referência" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="R$ #,##0.00"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -79,18 +79,8 @@
       <color rgb="00475569"/>
       <sz val="10"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="00000000"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="00333333"/>
-      <sz val="10"/>
-    </font>
   </fonts>
-  <fills count="13">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -137,21 +127,6 @@
         <fgColor rgb="00EDF1F7"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00CC0000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00166534"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00854D0E"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -179,7 +154,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -215,27 +190,6 @@
     <xf numFmtId="0" fontId="9" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -601,16 +555,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G104"/>
+  <dimension ref="A1:H104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -650,15 +605,20 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
+          <t>Setor de Trabalho *</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
           <t>Custo por Hora (R$) *</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Horas por Dia Útil *</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Ativo (SIM/NÃO) *</t>
         </is>
@@ -685,13 +645,18 @@
           <t>Eletricista Industrial</t>
         </is>
       </c>
-      <c r="E4" s="5" t="n">
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Montagem de Campo</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="n">
         <v>55</v>
       </c>
-      <c r="F4" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G4" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -702,11 +667,12 @@
       <c r="B5" s="7" t="n"/>
       <c r="C5" s="7" t="n"/>
       <c r="D5" s="6" t="n"/>
-      <c r="E5" s="8" t="n"/>
-      <c r="F5" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -717,11 +683,12 @@
       <c r="B6" s="7" t="n"/>
       <c r="C6" s="7" t="n"/>
       <c r="D6" s="6" t="n"/>
-      <c r="E6" s="8" t="n"/>
-      <c r="F6" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -732,11 +699,12 @@
       <c r="B7" s="7" t="n"/>
       <c r="C7" s="7" t="n"/>
       <c r="D7" s="6" t="n"/>
-      <c r="E7" s="8" t="n"/>
-      <c r="F7" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
+      <c r="E7" s="6" t="n"/>
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -747,11 +715,12 @@
       <c r="B8" s="7" t="n"/>
       <c r="C8" s="7" t="n"/>
       <c r="D8" s="6" t="n"/>
-      <c r="E8" s="8" t="n"/>
-      <c r="F8" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="8" t="n"/>
+      <c r="G8" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -762,11 +731,12 @@
       <c r="B9" s="7" t="n"/>
       <c r="C9" s="7" t="n"/>
       <c r="D9" s="6" t="n"/>
-      <c r="E9" s="8" t="n"/>
-      <c r="F9" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="8" t="n"/>
+      <c r="G9" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -777,11 +747,12 @@
       <c r="B10" s="7" t="n"/>
       <c r="C10" s="7" t="n"/>
       <c r="D10" s="6" t="n"/>
-      <c r="E10" s="8" t="n"/>
-      <c r="F10" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="8" t="n"/>
+      <c r="G10" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -792,11 +763,12 @@
       <c r="B11" s="7" t="n"/>
       <c r="C11" s="7" t="n"/>
       <c r="D11" s="6" t="n"/>
-      <c r="E11" s="8" t="n"/>
-      <c r="F11" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="8" t="n"/>
+      <c r="G11" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -807,11 +779,12 @@
       <c r="B12" s="7" t="n"/>
       <c r="C12" s="7" t="n"/>
       <c r="D12" s="6" t="n"/>
-      <c r="E12" s="8" t="n"/>
-      <c r="F12" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="8" t="n"/>
+      <c r="G12" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -822,11 +795,12 @@
       <c r="B13" s="7" t="n"/>
       <c r="C13" s="7" t="n"/>
       <c r="D13" s="6" t="n"/>
-      <c r="E13" s="8" t="n"/>
-      <c r="F13" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G13" s="6" t="inlineStr">
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="8" t="n"/>
+      <c r="G13" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -837,11 +811,12 @@
       <c r="B14" s="7" t="n"/>
       <c r="C14" s="7" t="n"/>
       <c r="D14" s="6" t="n"/>
-      <c r="E14" s="8" t="n"/>
-      <c r="F14" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G14" s="6" t="inlineStr">
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="8" t="n"/>
+      <c r="G14" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -852,11 +827,12 @@
       <c r="B15" s="7" t="n"/>
       <c r="C15" s="7" t="n"/>
       <c r="D15" s="6" t="n"/>
-      <c r="E15" s="8" t="n"/>
-      <c r="F15" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="8" t="n"/>
+      <c r="G15" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -867,11 +843,12 @@
       <c r="B16" s="7" t="n"/>
       <c r="C16" s="7" t="n"/>
       <c r="D16" s="6" t="n"/>
-      <c r="E16" s="8" t="n"/>
-      <c r="F16" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G16" s="6" t="inlineStr">
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="8" t="n"/>
+      <c r="G16" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -882,11 +859,12 @@
       <c r="B17" s="7" t="n"/>
       <c r="C17" s="7" t="n"/>
       <c r="D17" s="6" t="n"/>
-      <c r="E17" s="8" t="n"/>
-      <c r="F17" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G17" s="6" t="inlineStr">
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="8" t="n"/>
+      <c r="G17" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -897,11 +875,12 @@
       <c r="B18" s="7" t="n"/>
       <c r="C18" s="7" t="n"/>
       <c r="D18" s="6" t="n"/>
-      <c r="E18" s="8" t="n"/>
-      <c r="F18" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G18" s="6" t="inlineStr">
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="8" t="n"/>
+      <c r="G18" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -912,11 +891,12 @@
       <c r="B19" s="7" t="n"/>
       <c r="C19" s="7" t="n"/>
       <c r="D19" s="6" t="n"/>
-      <c r="E19" s="8" t="n"/>
-      <c r="F19" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G19" s="6" t="inlineStr">
+      <c r="E19" s="6" t="n"/>
+      <c r="F19" s="8" t="n"/>
+      <c r="G19" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -927,11 +907,12 @@
       <c r="B20" s="7" t="n"/>
       <c r="C20" s="7" t="n"/>
       <c r="D20" s="6" t="n"/>
-      <c r="E20" s="8" t="n"/>
-      <c r="F20" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G20" s="6" t="inlineStr">
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="8" t="n"/>
+      <c r="G20" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -942,11 +923,12 @@
       <c r="B21" s="7" t="n"/>
       <c r="C21" s="7" t="n"/>
       <c r="D21" s="6" t="n"/>
-      <c r="E21" s="8" t="n"/>
-      <c r="F21" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G21" s="6" t="inlineStr">
+      <c r="E21" s="6" t="n"/>
+      <c r="F21" s="8" t="n"/>
+      <c r="G21" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -957,11 +939,12 @@
       <c r="B22" s="7" t="n"/>
       <c r="C22" s="7" t="n"/>
       <c r="D22" s="6" t="n"/>
-      <c r="E22" s="8" t="n"/>
-      <c r="F22" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G22" s="6" t="inlineStr">
+      <c r="E22" s="6" t="n"/>
+      <c r="F22" s="8" t="n"/>
+      <c r="G22" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -972,11 +955,12 @@
       <c r="B23" s="7" t="n"/>
       <c r="C23" s="7" t="n"/>
       <c r="D23" s="6" t="n"/>
-      <c r="E23" s="8" t="n"/>
-      <c r="F23" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G23" s="6" t="inlineStr">
+      <c r="E23" s="6" t="n"/>
+      <c r="F23" s="8" t="n"/>
+      <c r="G23" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H23" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -987,11 +971,12 @@
       <c r="B24" s="7" t="n"/>
       <c r="C24" s="7" t="n"/>
       <c r="D24" s="6" t="n"/>
-      <c r="E24" s="8" t="n"/>
-      <c r="F24" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G24" s="6" t="inlineStr">
+      <c r="E24" s="6" t="n"/>
+      <c r="F24" s="8" t="n"/>
+      <c r="G24" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1002,11 +987,12 @@
       <c r="B25" s="7" t="n"/>
       <c r="C25" s="7" t="n"/>
       <c r="D25" s="6" t="n"/>
-      <c r="E25" s="8" t="n"/>
-      <c r="F25" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G25" s="6" t="inlineStr">
+      <c r="E25" s="6" t="n"/>
+      <c r="F25" s="8" t="n"/>
+      <c r="G25" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1017,11 +1003,12 @@
       <c r="B26" s="7" t="n"/>
       <c r="C26" s="7" t="n"/>
       <c r="D26" s="6" t="n"/>
-      <c r="E26" s="8" t="n"/>
-      <c r="F26" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G26" s="6" t="inlineStr">
+      <c r="E26" s="6" t="n"/>
+      <c r="F26" s="8" t="n"/>
+      <c r="G26" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1032,11 +1019,12 @@
       <c r="B27" s="7" t="n"/>
       <c r="C27" s="7" t="n"/>
       <c r="D27" s="6" t="n"/>
-      <c r="E27" s="8" t="n"/>
-      <c r="F27" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
+      <c r="E27" s="6" t="n"/>
+      <c r="F27" s="8" t="n"/>
+      <c r="G27" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1047,11 +1035,12 @@
       <c r="B28" s="7" t="n"/>
       <c r="C28" s="7" t="n"/>
       <c r="D28" s="6" t="n"/>
-      <c r="E28" s="8" t="n"/>
-      <c r="F28" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G28" s="6" t="inlineStr">
+      <c r="E28" s="6" t="n"/>
+      <c r="F28" s="8" t="n"/>
+      <c r="G28" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1062,11 +1051,12 @@
       <c r="B29" s="7" t="n"/>
       <c r="C29" s="7" t="n"/>
       <c r="D29" s="6" t="n"/>
-      <c r="E29" s="8" t="n"/>
-      <c r="F29" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G29" s="6" t="inlineStr">
+      <c r="E29" s="6" t="n"/>
+      <c r="F29" s="8" t="n"/>
+      <c r="G29" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H29" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1077,11 +1067,12 @@
       <c r="B30" s="7" t="n"/>
       <c r="C30" s="7" t="n"/>
       <c r="D30" s="6" t="n"/>
-      <c r="E30" s="8" t="n"/>
-      <c r="F30" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G30" s="6" t="inlineStr">
+      <c r="E30" s="6" t="n"/>
+      <c r="F30" s="8" t="n"/>
+      <c r="G30" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H30" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1092,11 +1083,12 @@
       <c r="B31" s="7" t="n"/>
       <c r="C31" s="7" t="n"/>
       <c r="D31" s="6" t="n"/>
-      <c r="E31" s="8" t="n"/>
-      <c r="F31" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G31" s="6" t="inlineStr">
+      <c r="E31" s="6" t="n"/>
+      <c r="F31" s="8" t="n"/>
+      <c r="G31" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H31" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1107,11 +1099,12 @@
       <c r="B32" s="7" t="n"/>
       <c r="C32" s="7" t="n"/>
       <c r="D32" s="6" t="n"/>
-      <c r="E32" s="8" t="n"/>
-      <c r="F32" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G32" s="6" t="inlineStr">
+      <c r="E32" s="6" t="n"/>
+      <c r="F32" s="8" t="n"/>
+      <c r="G32" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H32" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1122,11 +1115,12 @@
       <c r="B33" s="7" t="n"/>
       <c r="C33" s="7" t="n"/>
       <c r="D33" s="6" t="n"/>
-      <c r="E33" s="8" t="n"/>
-      <c r="F33" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G33" s="6" t="inlineStr">
+      <c r="E33" s="6" t="n"/>
+      <c r="F33" s="8" t="n"/>
+      <c r="G33" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H33" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1137,11 +1131,12 @@
       <c r="B34" s="7" t="n"/>
       <c r="C34" s="7" t="n"/>
       <c r="D34" s="6" t="n"/>
-      <c r="E34" s="8" t="n"/>
-      <c r="F34" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G34" s="6" t="inlineStr">
+      <c r="E34" s="6" t="n"/>
+      <c r="F34" s="8" t="n"/>
+      <c r="G34" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H34" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1152,11 +1147,12 @@
       <c r="B35" s="7" t="n"/>
       <c r="C35" s="7" t="n"/>
       <c r="D35" s="6" t="n"/>
-      <c r="E35" s="8" t="n"/>
-      <c r="F35" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G35" s="6" t="inlineStr">
+      <c r="E35" s="6" t="n"/>
+      <c r="F35" s="8" t="n"/>
+      <c r="G35" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H35" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1167,11 +1163,12 @@
       <c r="B36" s="7" t="n"/>
       <c r="C36" s="7" t="n"/>
       <c r="D36" s="6" t="n"/>
-      <c r="E36" s="8" t="n"/>
-      <c r="F36" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G36" s="6" t="inlineStr">
+      <c r="E36" s="6" t="n"/>
+      <c r="F36" s="8" t="n"/>
+      <c r="G36" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H36" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1182,11 +1179,12 @@
       <c r="B37" s="7" t="n"/>
       <c r="C37" s="7" t="n"/>
       <c r="D37" s="6" t="n"/>
-      <c r="E37" s="8" t="n"/>
-      <c r="F37" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G37" s="6" t="inlineStr">
+      <c r="E37" s="6" t="n"/>
+      <c r="F37" s="8" t="n"/>
+      <c r="G37" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H37" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1197,11 +1195,12 @@
       <c r="B38" s="7" t="n"/>
       <c r="C38" s="7" t="n"/>
       <c r="D38" s="6" t="n"/>
-      <c r="E38" s="8" t="n"/>
-      <c r="F38" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G38" s="6" t="inlineStr">
+      <c r="E38" s="6" t="n"/>
+      <c r="F38" s="8" t="n"/>
+      <c r="G38" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H38" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1212,11 +1211,12 @@
       <c r="B39" s="7" t="n"/>
       <c r="C39" s="7" t="n"/>
       <c r="D39" s="6" t="n"/>
-      <c r="E39" s="8" t="n"/>
-      <c r="F39" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G39" s="6" t="inlineStr">
+      <c r="E39" s="6" t="n"/>
+      <c r="F39" s="8" t="n"/>
+      <c r="G39" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H39" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1227,11 +1227,12 @@
       <c r="B40" s="7" t="n"/>
       <c r="C40" s="7" t="n"/>
       <c r="D40" s="6" t="n"/>
-      <c r="E40" s="8" t="n"/>
-      <c r="F40" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G40" s="6" t="inlineStr">
+      <c r="E40" s="6" t="n"/>
+      <c r="F40" s="8" t="n"/>
+      <c r="G40" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H40" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1242,11 +1243,12 @@
       <c r="B41" s="7" t="n"/>
       <c r="C41" s="7" t="n"/>
       <c r="D41" s="6" t="n"/>
-      <c r="E41" s="8" t="n"/>
-      <c r="F41" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G41" s="6" t="inlineStr">
+      <c r="E41" s="6" t="n"/>
+      <c r="F41" s="8" t="n"/>
+      <c r="G41" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H41" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1257,11 +1259,12 @@
       <c r="B42" s="7" t="n"/>
       <c r="C42" s="7" t="n"/>
       <c r="D42" s="6" t="n"/>
-      <c r="E42" s="8" t="n"/>
-      <c r="F42" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G42" s="6" t="inlineStr">
+      <c r="E42" s="6" t="n"/>
+      <c r="F42" s="8" t="n"/>
+      <c r="G42" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H42" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1272,11 +1275,12 @@
       <c r="B43" s="7" t="n"/>
       <c r="C43" s="7" t="n"/>
       <c r="D43" s="6" t="n"/>
-      <c r="E43" s="8" t="n"/>
-      <c r="F43" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G43" s="6" t="inlineStr">
+      <c r="E43" s="6" t="n"/>
+      <c r="F43" s="8" t="n"/>
+      <c r="G43" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H43" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1287,11 +1291,12 @@
       <c r="B44" s="7" t="n"/>
       <c r="C44" s="7" t="n"/>
       <c r="D44" s="6" t="n"/>
-      <c r="E44" s="8" t="n"/>
-      <c r="F44" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G44" s="6" t="inlineStr">
+      <c r="E44" s="6" t="n"/>
+      <c r="F44" s="8" t="n"/>
+      <c r="G44" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H44" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1302,11 +1307,12 @@
       <c r="B45" s="7" t="n"/>
       <c r="C45" s="7" t="n"/>
       <c r="D45" s="6" t="n"/>
-      <c r="E45" s="8" t="n"/>
-      <c r="F45" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G45" s="6" t="inlineStr">
+      <c r="E45" s="6" t="n"/>
+      <c r="F45" s="8" t="n"/>
+      <c r="G45" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H45" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1317,11 +1323,12 @@
       <c r="B46" s="7" t="n"/>
       <c r="C46" s="7" t="n"/>
       <c r="D46" s="6" t="n"/>
-      <c r="E46" s="8" t="n"/>
-      <c r="F46" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G46" s="6" t="inlineStr">
+      <c r="E46" s="6" t="n"/>
+      <c r="F46" s="8" t="n"/>
+      <c r="G46" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H46" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1332,11 +1339,12 @@
       <c r="B47" s="7" t="n"/>
       <c r="C47" s="7" t="n"/>
       <c r="D47" s="6" t="n"/>
-      <c r="E47" s="8" t="n"/>
-      <c r="F47" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G47" s="6" t="inlineStr">
+      <c r="E47" s="6" t="n"/>
+      <c r="F47" s="8" t="n"/>
+      <c r="G47" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H47" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1347,11 +1355,12 @@
       <c r="B48" s="7" t="n"/>
       <c r="C48" s="7" t="n"/>
       <c r="D48" s="6" t="n"/>
-      <c r="E48" s="8" t="n"/>
-      <c r="F48" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G48" s="6" t="inlineStr">
+      <c r="E48" s="6" t="n"/>
+      <c r="F48" s="8" t="n"/>
+      <c r="G48" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H48" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1362,11 +1371,12 @@
       <c r="B49" s="7" t="n"/>
       <c r="C49" s="7" t="n"/>
       <c r="D49" s="6" t="n"/>
-      <c r="E49" s="8" t="n"/>
-      <c r="F49" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G49" s="6" t="inlineStr">
+      <c r="E49" s="6" t="n"/>
+      <c r="F49" s="8" t="n"/>
+      <c r="G49" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H49" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1377,11 +1387,12 @@
       <c r="B50" s="7" t="n"/>
       <c r="C50" s="7" t="n"/>
       <c r="D50" s="6" t="n"/>
-      <c r="E50" s="8" t="n"/>
-      <c r="F50" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G50" s="6" t="inlineStr">
+      <c r="E50" s="6" t="n"/>
+      <c r="F50" s="8" t="n"/>
+      <c r="G50" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H50" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1392,11 +1403,12 @@
       <c r="B51" s="7" t="n"/>
       <c r="C51" s="7" t="n"/>
       <c r="D51" s="6" t="n"/>
-      <c r="E51" s="8" t="n"/>
-      <c r="F51" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G51" s="6" t="inlineStr">
+      <c r="E51" s="6" t="n"/>
+      <c r="F51" s="8" t="n"/>
+      <c r="G51" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H51" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1407,11 +1419,12 @@
       <c r="B52" s="7" t="n"/>
       <c r="C52" s="7" t="n"/>
       <c r="D52" s="6" t="n"/>
-      <c r="E52" s="8" t="n"/>
-      <c r="F52" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G52" s="6" t="inlineStr">
+      <c r="E52" s="6" t="n"/>
+      <c r="F52" s="8" t="n"/>
+      <c r="G52" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H52" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1422,11 +1435,12 @@
       <c r="B53" s="7" t="n"/>
       <c r="C53" s="7" t="n"/>
       <c r="D53" s="6" t="n"/>
-      <c r="E53" s="8" t="n"/>
-      <c r="F53" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G53" s="6" t="inlineStr">
+      <c r="E53" s="6" t="n"/>
+      <c r="F53" s="8" t="n"/>
+      <c r="G53" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H53" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1437,11 +1451,12 @@
       <c r="B54" s="7" t="n"/>
       <c r="C54" s="7" t="n"/>
       <c r="D54" s="6" t="n"/>
-      <c r="E54" s="8" t="n"/>
-      <c r="F54" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G54" s="6" t="inlineStr">
+      <c r="E54" s="6" t="n"/>
+      <c r="F54" s="8" t="n"/>
+      <c r="G54" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H54" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1452,11 +1467,12 @@
       <c r="B55" s="7" t="n"/>
       <c r="C55" s="7" t="n"/>
       <c r="D55" s="6" t="n"/>
-      <c r="E55" s="8" t="n"/>
-      <c r="F55" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G55" s="6" t="inlineStr">
+      <c r="E55" s="6" t="n"/>
+      <c r="F55" s="8" t="n"/>
+      <c r="G55" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H55" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1467,11 +1483,12 @@
       <c r="B56" s="7" t="n"/>
       <c r="C56" s="7" t="n"/>
       <c r="D56" s="6" t="n"/>
-      <c r="E56" s="8" t="n"/>
-      <c r="F56" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G56" s="6" t="inlineStr">
+      <c r="E56" s="6" t="n"/>
+      <c r="F56" s="8" t="n"/>
+      <c r="G56" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H56" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1482,11 +1499,12 @@
       <c r="B57" s="7" t="n"/>
       <c r="C57" s="7" t="n"/>
       <c r="D57" s="6" t="n"/>
-      <c r="E57" s="8" t="n"/>
-      <c r="F57" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G57" s="6" t="inlineStr">
+      <c r="E57" s="6" t="n"/>
+      <c r="F57" s="8" t="n"/>
+      <c r="G57" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H57" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1497,11 +1515,12 @@
       <c r="B58" s="7" t="n"/>
       <c r="C58" s="7" t="n"/>
       <c r="D58" s="6" t="n"/>
-      <c r="E58" s="8" t="n"/>
-      <c r="F58" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G58" s="6" t="inlineStr">
+      <c r="E58" s="6" t="n"/>
+      <c r="F58" s="8" t="n"/>
+      <c r="G58" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H58" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1512,11 +1531,12 @@
       <c r="B59" s="7" t="n"/>
       <c r="C59" s="7" t="n"/>
       <c r="D59" s="6" t="n"/>
-      <c r="E59" s="8" t="n"/>
-      <c r="F59" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G59" s="6" t="inlineStr">
+      <c r="E59" s="6" t="n"/>
+      <c r="F59" s="8" t="n"/>
+      <c r="G59" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H59" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1527,11 +1547,12 @@
       <c r="B60" s="7" t="n"/>
       <c r="C60" s="7" t="n"/>
       <c r="D60" s="6" t="n"/>
-      <c r="E60" s="8" t="n"/>
-      <c r="F60" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G60" s="6" t="inlineStr">
+      <c r="E60" s="6" t="n"/>
+      <c r="F60" s="8" t="n"/>
+      <c r="G60" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H60" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1542,11 +1563,12 @@
       <c r="B61" s="7" t="n"/>
       <c r="C61" s="7" t="n"/>
       <c r="D61" s="6" t="n"/>
-      <c r="E61" s="8" t="n"/>
-      <c r="F61" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G61" s="6" t="inlineStr">
+      <c r="E61" s="6" t="n"/>
+      <c r="F61" s="8" t="n"/>
+      <c r="G61" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H61" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1557,11 +1579,12 @@
       <c r="B62" s="7" t="n"/>
       <c r="C62" s="7" t="n"/>
       <c r="D62" s="6" t="n"/>
-      <c r="E62" s="8" t="n"/>
-      <c r="F62" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G62" s="6" t="inlineStr">
+      <c r="E62" s="6" t="n"/>
+      <c r="F62" s="8" t="n"/>
+      <c r="G62" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H62" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1572,11 +1595,12 @@
       <c r="B63" s="7" t="n"/>
       <c r="C63" s="7" t="n"/>
       <c r="D63" s="6" t="n"/>
-      <c r="E63" s="8" t="n"/>
-      <c r="F63" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G63" s="6" t="inlineStr">
+      <c r="E63" s="6" t="n"/>
+      <c r="F63" s="8" t="n"/>
+      <c r="G63" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H63" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1587,11 +1611,12 @@
       <c r="B64" s="7" t="n"/>
       <c r="C64" s="7" t="n"/>
       <c r="D64" s="6" t="n"/>
-      <c r="E64" s="8" t="n"/>
-      <c r="F64" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G64" s="6" t="inlineStr">
+      <c r="E64" s="6" t="n"/>
+      <c r="F64" s="8" t="n"/>
+      <c r="G64" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H64" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1602,11 +1627,12 @@
       <c r="B65" s="7" t="n"/>
       <c r="C65" s="7" t="n"/>
       <c r="D65" s="6" t="n"/>
-      <c r="E65" s="8" t="n"/>
-      <c r="F65" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G65" s="6" t="inlineStr">
+      <c r="E65" s="6" t="n"/>
+      <c r="F65" s="8" t="n"/>
+      <c r="G65" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H65" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1617,11 +1643,12 @@
       <c r="B66" s="7" t="n"/>
       <c r="C66" s="7" t="n"/>
       <c r="D66" s="6" t="n"/>
-      <c r="E66" s="8" t="n"/>
-      <c r="F66" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G66" s="6" t="inlineStr">
+      <c r="E66" s="6" t="n"/>
+      <c r="F66" s="8" t="n"/>
+      <c r="G66" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H66" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1632,11 +1659,12 @@
       <c r="B67" s="7" t="n"/>
       <c r="C67" s="7" t="n"/>
       <c r="D67" s="6" t="n"/>
-      <c r="E67" s="8" t="n"/>
-      <c r="F67" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G67" s="6" t="inlineStr">
+      <c r="E67" s="6" t="n"/>
+      <c r="F67" s="8" t="n"/>
+      <c r="G67" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H67" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1647,11 +1675,12 @@
       <c r="B68" s="7" t="n"/>
       <c r="C68" s="7" t="n"/>
       <c r="D68" s="6" t="n"/>
-      <c r="E68" s="8" t="n"/>
-      <c r="F68" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G68" s="6" t="inlineStr">
+      <c r="E68" s="6" t="n"/>
+      <c r="F68" s="8" t="n"/>
+      <c r="G68" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H68" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1662,11 +1691,12 @@
       <c r="B69" s="7" t="n"/>
       <c r="C69" s="7" t="n"/>
       <c r="D69" s="6" t="n"/>
-      <c r="E69" s="8" t="n"/>
-      <c r="F69" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G69" s="6" t="inlineStr">
+      <c r="E69" s="6" t="n"/>
+      <c r="F69" s="8" t="n"/>
+      <c r="G69" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H69" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1677,11 +1707,12 @@
       <c r="B70" s="7" t="n"/>
       <c r="C70" s="7" t="n"/>
       <c r="D70" s="6" t="n"/>
-      <c r="E70" s="8" t="n"/>
-      <c r="F70" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G70" s="6" t="inlineStr">
+      <c r="E70" s="6" t="n"/>
+      <c r="F70" s="8" t="n"/>
+      <c r="G70" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H70" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1692,11 +1723,12 @@
       <c r="B71" s="7" t="n"/>
       <c r="C71" s="7" t="n"/>
       <c r="D71" s="6" t="n"/>
-      <c r="E71" s="8" t="n"/>
-      <c r="F71" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G71" s="6" t="inlineStr">
+      <c r="E71" s="6" t="n"/>
+      <c r="F71" s="8" t="n"/>
+      <c r="G71" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H71" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1707,11 +1739,12 @@
       <c r="B72" s="7" t="n"/>
       <c r="C72" s="7" t="n"/>
       <c r="D72" s="6" t="n"/>
-      <c r="E72" s="8" t="n"/>
-      <c r="F72" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G72" s="6" t="inlineStr">
+      <c r="E72" s="6" t="n"/>
+      <c r="F72" s="8" t="n"/>
+      <c r="G72" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H72" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1722,11 +1755,12 @@
       <c r="B73" s="7" t="n"/>
       <c r="C73" s="7" t="n"/>
       <c r="D73" s="6" t="n"/>
-      <c r="E73" s="8" t="n"/>
-      <c r="F73" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G73" s="6" t="inlineStr">
+      <c r="E73" s="6" t="n"/>
+      <c r="F73" s="8" t="n"/>
+      <c r="G73" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H73" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1737,11 +1771,12 @@
       <c r="B74" s="7" t="n"/>
       <c r="C74" s="7" t="n"/>
       <c r="D74" s="6" t="n"/>
-      <c r="E74" s="8" t="n"/>
-      <c r="F74" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G74" s="6" t="inlineStr">
+      <c r="E74" s="6" t="n"/>
+      <c r="F74" s="8" t="n"/>
+      <c r="G74" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H74" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1752,11 +1787,12 @@
       <c r="B75" s="7" t="n"/>
       <c r="C75" s="7" t="n"/>
       <c r="D75" s="6" t="n"/>
-      <c r="E75" s="8" t="n"/>
-      <c r="F75" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G75" s="6" t="inlineStr">
+      <c r="E75" s="6" t="n"/>
+      <c r="F75" s="8" t="n"/>
+      <c r="G75" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H75" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1767,11 +1803,12 @@
       <c r="B76" s="7" t="n"/>
       <c r="C76" s="7" t="n"/>
       <c r="D76" s="6" t="n"/>
-      <c r="E76" s="8" t="n"/>
-      <c r="F76" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G76" s="6" t="inlineStr">
+      <c r="E76" s="6" t="n"/>
+      <c r="F76" s="8" t="n"/>
+      <c r="G76" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H76" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1782,11 +1819,12 @@
       <c r="B77" s="7" t="n"/>
       <c r="C77" s="7" t="n"/>
       <c r="D77" s="6" t="n"/>
-      <c r="E77" s="8" t="n"/>
-      <c r="F77" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G77" s="6" t="inlineStr">
+      <c r="E77" s="6" t="n"/>
+      <c r="F77" s="8" t="n"/>
+      <c r="G77" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H77" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1797,11 +1835,12 @@
       <c r="B78" s="7" t="n"/>
       <c r="C78" s="7" t="n"/>
       <c r="D78" s="6" t="n"/>
-      <c r="E78" s="8" t="n"/>
-      <c r="F78" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G78" s="6" t="inlineStr">
+      <c r="E78" s="6" t="n"/>
+      <c r="F78" s="8" t="n"/>
+      <c r="G78" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H78" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1812,11 +1851,12 @@
       <c r="B79" s="7" t="n"/>
       <c r="C79" s="7" t="n"/>
       <c r="D79" s="6" t="n"/>
-      <c r="E79" s="8" t="n"/>
-      <c r="F79" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G79" s="6" t="inlineStr">
+      <c r="E79" s="6" t="n"/>
+      <c r="F79" s="8" t="n"/>
+      <c r="G79" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H79" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1827,11 +1867,12 @@
       <c r="B80" s="7" t="n"/>
       <c r="C80" s="7" t="n"/>
       <c r="D80" s="6" t="n"/>
-      <c r="E80" s="8" t="n"/>
-      <c r="F80" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G80" s="6" t="inlineStr">
+      <c r="E80" s="6" t="n"/>
+      <c r="F80" s="8" t="n"/>
+      <c r="G80" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H80" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1842,11 +1883,12 @@
       <c r="B81" s="7" t="n"/>
       <c r="C81" s="7" t="n"/>
       <c r="D81" s="6" t="n"/>
-      <c r="E81" s="8" t="n"/>
-      <c r="F81" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G81" s="6" t="inlineStr">
+      <c r="E81" s="6" t="n"/>
+      <c r="F81" s="8" t="n"/>
+      <c r="G81" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H81" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1857,11 +1899,12 @@
       <c r="B82" s="7" t="n"/>
       <c r="C82" s="7" t="n"/>
       <c r="D82" s="6" t="n"/>
-      <c r="E82" s="8" t="n"/>
-      <c r="F82" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G82" s="6" t="inlineStr">
+      <c r="E82" s="6" t="n"/>
+      <c r="F82" s="8" t="n"/>
+      <c r="G82" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H82" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1872,11 +1915,12 @@
       <c r="B83" s="7" t="n"/>
       <c r="C83" s="7" t="n"/>
       <c r="D83" s="6" t="n"/>
-      <c r="E83" s="8" t="n"/>
-      <c r="F83" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G83" s="6" t="inlineStr">
+      <c r="E83" s="6" t="n"/>
+      <c r="F83" s="8" t="n"/>
+      <c r="G83" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H83" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1887,11 +1931,12 @@
       <c r="B84" s="7" t="n"/>
       <c r="C84" s="7" t="n"/>
       <c r="D84" s="6" t="n"/>
-      <c r="E84" s="8" t="n"/>
-      <c r="F84" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G84" s="6" t="inlineStr">
+      <c r="E84" s="6" t="n"/>
+      <c r="F84" s="8" t="n"/>
+      <c r="G84" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H84" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1902,11 +1947,12 @@
       <c r="B85" s="7" t="n"/>
       <c r="C85" s="7" t="n"/>
       <c r="D85" s="6" t="n"/>
-      <c r="E85" s="8" t="n"/>
-      <c r="F85" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G85" s="6" t="inlineStr">
+      <c r="E85" s="6" t="n"/>
+      <c r="F85" s="8" t="n"/>
+      <c r="G85" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H85" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1917,11 +1963,12 @@
       <c r="B86" s="7" t="n"/>
       <c r="C86" s="7" t="n"/>
       <c r="D86" s="6" t="n"/>
-      <c r="E86" s="8" t="n"/>
-      <c r="F86" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G86" s="6" t="inlineStr">
+      <c r="E86" s="6" t="n"/>
+      <c r="F86" s="8" t="n"/>
+      <c r="G86" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H86" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1932,11 +1979,12 @@
       <c r="B87" s="7" t="n"/>
       <c r="C87" s="7" t="n"/>
       <c r="D87" s="6" t="n"/>
-      <c r="E87" s="8" t="n"/>
-      <c r="F87" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G87" s="6" t="inlineStr">
+      <c r="E87" s="6" t="n"/>
+      <c r="F87" s="8" t="n"/>
+      <c r="G87" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H87" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1947,11 +1995,12 @@
       <c r="B88" s="7" t="n"/>
       <c r="C88" s="7" t="n"/>
       <c r="D88" s="6" t="n"/>
-      <c r="E88" s="8" t="n"/>
-      <c r="F88" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G88" s="6" t="inlineStr">
+      <c r="E88" s="6" t="n"/>
+      <c r="F88" s="8" t="n"/>
+      <c r="G88" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H88" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1962,11 +2011,12 @@
       <c r="B89" s="7" t="n"/>
       <c r="C89" s="7" t="n"/>
       <c r="D89" s="6" t="n"/>
-      <c r="E89" s="8" t="n"/>
-      <c r="F89" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G89" s="6" t="inlineStr">
+      <c r="E89" s="6" t="n"/>
+      <c r="F89" s="8" t="n"/>
+      <c r="G89" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H89" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1977,11 +2027,12 @@
       <c r="B90" s="7" t="n"/>
       <c r="C90" s="7" t="n"/>
       <c r="D90" s="6" t="n"/>
-      <c r="E90" s="8" t="n"/>
-      <c r="F90" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G90" s="6" t="inlineStr">
+      <c r="E90" s="6" t="n"/>
+      <c r="F90" s="8" t="n"/>
+      <c r="G90" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H90" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -1992,11 +2043,12 @@
       <c r="B91" s="7" t="n"/>
       <c r="C91" s="7" t="n"/>
       <c r="D91" s="6" t="n"/>
-      <c r="E91" s="8" t="n"/>
-      <c r="F91" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G91" s="6" t="inlineStr">
+      <c r="E91" s="6" t="n"/>
+      <c r="F91" s="8" t="n"/>
+      <c r="G91" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H91" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -2007,11 +2059,12 @@
       <c r="B92" s="7" t="n"/>
       <c r="C92" s="7" t="n"/>
       <c r="D92" s="6" t="n"/>
-      <c r="E92" s="8" t="n"/>
-      <c r="F92" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G92" s="6" t="inlineStr">
+      <c r="E92" s="6" t="n"/>
+      <c r="F92" s="8" t="n"/>
+      <c r="G92" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H92" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -2022,11 +2075,12 @@
       <c r="B93" s="7" t="n"/>
       <c r="C93" s="7" t="n"/>
       <c r="D93" s="6" t="n"/>
-      <c r="E93" s="8" t="n"/>
-      <c r="F93" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G93" s="6" t="inlineStr">
+      <c r="E93" s="6" t="n"/>
+      <c r="F93" s="8" t="n"/>
+      <c r="G93" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H93" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -2037,11 +2091,12 @@
       <c r="B94" s="7" t="n"/>
       <c r="C94" s="7" t="n"/>
       <c r="D94" s="6" t="n"/>
-      <c r="E94" s="8" t="n"/>
-      <c r="F94" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G94" s="6" t="inlineStr">
+      <c r="E94" s="6" t="n"/>
+      <c r="F94" s="8" t="n"/>
+      <c r="G94" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H94" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -2052,11 +2107,12 @@
       <c r="B95" s="7" t="n"/>
       <c r="C95" s="7" t="n"/>
       <c r="D95" s="6" t="n"/>
-      <c r="E95" s="8" t="n"/>
-      <c r="F95" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G95" s="6" t="inlineStr">
+      <c r="E95" s="6" t="n"/>
+      <c r="F95" s="8" t="n"/>
+      <c r="G95" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H95" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -2067,11 +2123,12 @@
       <c r="B96" s="7" t="n"/>
       <c r="C96" s="7" t="n"/>
       <c r="D96" s="6" t="n"/>
-      <c r="E96" s="8" t="n"/>
-      <c r="F96" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G96" s="6" t="inlineStr">
+      <c r="E96" s="6" t="n"/>
+      <c r="F96" s="8" t="n"/>
+      <c r="G96" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H96" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -2082,11 +2139,12 @@
       <c r="B97" s="7" t="n"/>
       <c r="C97" s="7" t="n"/>
       <c r="D97" s="6" t="n"/>
-      <c r="E97" s="8" t="n"/>
-      <c r="F97" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G97" s="6" t="inlineStr">
+      <c r="E97" s="6" t="n"/>
+      <c r="F97" s="8" t="n"/>
+      <c r="G97" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H97" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -2097,11 +2155,12 @@
       <c r="B98" s="7" t="n"/>
       <c r="C98" s="7" t="n"/>
       <c r="D98" s="6" t="n"/>
-      <c r="E98" s="8" t="n"/>
-      <c r="F98" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G98" s="6" t="inlineStr">
+      <c r="E98" s="6" t="n"/>
+      <c r="F98" s="8" t="n"/>
+      <c r="G98" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H98" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -2112,11 +2171,12 @@
       <c r="B99" s="7" t="n"/>
       <c r="C99" s="7" t="n"/>
       <c r="D99" s="6" t="n"/>
-      <c r="E99" s="8" t="n"/>
-      <c r="F99" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G99" s="6" t="inlineStr">
+      <c r="E99" s="6" t="n"/>
+      <c r="F99" s="8" t="n"/>
+      <c r="G99" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H99" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -2127,11 +2187,12 @@
       <c r="B100" s="7" t="n"/>
       <c r="C100" s="7" t="n"/>
       <c r="D100" s="6" t="n"/>
-      <c r="E100" s="8" t="n"/>
-      <c r="F100" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G100" s="6" t="inlineStr">
+      <c r="E100" s="6" t="n"/>
+      <c r="F100" s="8" t="n"/>
+      <c r="G100" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H100" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -2142,11 +2203,12 @@
       <c r="B101" s="7" t="n"/>
       <c r="C101" s="7" t="n"/>
       <c r="D101" s="6" t="n"/>
-      <c r="E101" s="8" t="n"/>
-      <c r="F101" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G101" s="6" t="inlineStr">
+      <c r="E101" s="6" t="n"/>
+      <c r="F101" s="8" t="n"/>
+      <c r="G101" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H101" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -2157,11 +2219,12 @@
       <c r="B102" s="7" t="n"/>
       <c r="C102" s="7" t="n"/>
       <c r="D102" s="6" t="n"/>
-      <c r="E102" s="8" t="n"/>
-      <c r="F102" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G102" s="6" t="inlineStr">
+      <c r="E102" s="6" t="n"/>
+      <c r="F102" s="8" t="n"/>
+      <c r="G102" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H102" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -2172,11 +2235,12 @@
       <c r="B103" s="7" t="n"/>
       <c r="C103" s="7" t="n"/>
       <c r="D103" s="6" t="n"/>
-      <c r="E103" s="8" t="n"/>
-      <c r="F103" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G103" s="6" t="inlineStr">
+      <c r="E103" s="6" t="n"/>
+      <c r="F103" s="8" t="n"/>
+      <c r="G103" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H103" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -2187,11 +2251,12 @@
       <c r="B104" s="7" t="n"/>
       <c r="C104" s="7" t="n"/>
       <c r="D104" s="6" t="n"/>
-      <c r="E104" s="8" t="n"/>
-      <c r="F104" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G104" s="6" t="inlineStr">
+      <c r="E104" s="6" t="n"/>
+      <c r="F104" s="8" t="n"/>
+      <c r="G104" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="H104" s="6" t="inlineStr">
         <is>
           <t>SIM</t>
         </is>
@@ -2199,19 +2264,19 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <dataValidations count="3">
-    <dataValidation sqref="G5:G104" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Valor inválido" error="Digite SIM ou NÃO" type="list">
+    <dataValidation sqref="H5:H104" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Valor inválido" error="Digite SIM ou NÃO" type="list">
       <formula1>"SIM,NÃO"</formula1>
     </dataValidation>
-    <dataValidation sqref="F5:F104" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Horas inválidas" error="Digite entre 1 e 24" type="decimal" operator="between">
+    <dataValidation sqref="G5:G104" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Horas inválidas" error="Entre 1 e 24" type="decimal" operator="between">
       <formula1>1</formula1>
       <formula2>24</formula2>
     </dataValidation>
-    <dataValidation sqref="E5:E104" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Custo inválido" error="Digite um valor &gt;= 0" type="decimal" operator="greaterThanOrEqual">
-      <formula1>0</formula1>
+    <dataValidation sqref="E5:E104" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Engenharia Elétrica,Engenharia de Software,Engenharia de Automação,Projetos,Montagem de Painel,Montagem de Campo,Comissionamento,Manutenção,Administrativo,Suporte Técnico"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2224,245 +2289,149 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="9" t="inlineStr">
         <is>
-          <t>Cargos / Funções Sugeridos</t>
+          <t>Setores de Trabalho Disponíveis</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>Cargo / Função</t>
+          <t>Setor de Trabalho</t>
         </is>
       </c>
       <c r="B2" s="10" t="inlineStr">
         <is>
-          <t>Área</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
+          <t>Descrição</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="16" customHeight="1">
       <c r="A3" s="11" t="inlineStr">
         <is>
-          <t>Engenheiro Eletricista</t>
+          <t>Engenharia Elétrica</t>
         </is>
       </c>
       <c r="B3" s="12" t="inlineStr">
         <is>
-          <t>Engenharia</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
+          <t>Projetos e especificações elétricas, dimensionamentos</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="16" customHeight="1">
       <c r="A4" s="13" t="inlineStr">
         <is>
-          <t>Engenheiro de Automação</t>
+          <t>Engenharia de Software</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>Engenharia</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
+          <t>Desenvolvimento de sistemas, SCADA, interfaces</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="16" customHeight="1">
       <c r="A5" s="11" t="inlineStr">
         <is>
-          <t>Técnico em Automação</t>
+          <t>Engenharia de Automação</t>
         </is>
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Técnico</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
+          <t>CLPs, redes industriais, programação de automação</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16" customHeight="1">
       <c r="A6" s="13" t="inlineStr">
         <is>
-          <t>Técnico Eletrotécnico</t>
+          <t>Projetos</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>Técnico</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
+          <t>Documentação técnica, desenhos, diagramas</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="16" customHeight="1">
       <c r="A7" s="11" t="inlineStr">
         <is>
-          <t>Técnico de Campo</t>
+          <t>Montagem de Painel</t>
         </is>
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>Técnico</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
+          <t>Montagem física de painéis elétricos e CCMs</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="16" customHeight="1">
       <c r="A8" s="13" t="inlineStr">
         <is>
-          <t>Eletricista Industrial</t>
+          <t>Montagem de Campo</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>Execução</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
+          <t>Instalação elétrica em campo, cabeamento</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="16" customHeight="1">
       <c r="A9" s="11" t="inlineStr">
         <is>
-          <t>Eletricista Instalador</t>
+          <t>Comissionamento</t>
         </is>
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>Execução</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
+          <t>Testes, start-up e comissionamento de sistemas</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="16" customHeight="1">
       <c r="A10" s="13" t="inlineStr">
         <is>
-          <t>Auxiliar Elétrico</t>
+          <t>Manutenção</t>
         </is>
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>Execução</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
+          <t>Manutenção preventiva e corretiva</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="16" customHeight="1">
       <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>Programador CLP</t>
+          <t>Suporte Técnico</t>
         </is>
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>Automação</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
+          <t>Suporte remoto e presencial pós-obra</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="16" customHeight="1">
       <c r="A12" s="13" t="inlineStr">
         <is>
-          <t>Programador SCADA</t>
+          <t>Administrativo</t>
         </is>
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>Automação</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="11" t="inlineStr">
-        <is>
-          <t>Projetista Elétrico</t>
-        </is>
-      </c>
-      <c r="B13" s="12" t="inlineStr">
-        <is>
-          <t>Projetos</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="13" t="inlineStr">
-        <is>
-          <t>Desenhista CAD</t>
-        </is>
-      </c>
-      <c r="B14" s="14" t="inlineStr">
-        <is>
-          <t>Projetos</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="11" t="inlineStr">
-        <is>
-          <t>Supervisor de Obras</t>
-        </is>
-      </c>
-      <c r="B15" s="12" t="inlineStr">
-        <is>
-          <t>Gestão</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="13" t="inlineStr">
-        <is>
-          <t>Encarregado de Obras</t>
-        </is>
-      </c>
-      <c r="B16" s="14" t="inlineStr">
-        <is>
-          <t>Gestão</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="11" t="inlineStr">
-        <is>
-          <t>Assistente Técnico</t>
-        </is>
-      </c>
-      <c r="B17" s="12" t="inlineStr">
-        <is>
-          <t>Suporte</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="13" t="inlineStr">
-        <is>
-          <t>Operador de Painel</t>
-        </is>
-      </c>
-      <c r="B18" s="14" t="inlineStr">
-        <is>
-          <t>Operação</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="11" t="inlineStr">
-        <is>
-          <t>Gerente de Projetos</t>
-        </is>
-      </c>
-      <c r="B19" s="12" t="inlineStr">
-        <is>
-          <t>Gestão</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="13" t="inlineStr">
-        <is>
-          <t>Coordenador de Automação</t>
-        </is>
-      </c>
-      <c r="B20" s="14" t="inlineStr">
-        <is>
-          <t>Gestão</t>
+          <t>Gestão administrativa, compras, logística</t>
         </is>
       </c>
     </row>
@@ -2480,165 +2449,228 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A24"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="85" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="15" t="inlineStr">
-        <is>
-          <t>INSTRUÇÕES DE PREENCHIMENTO</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="6" customHeight="1">
-      <c r="A2" s="16" t="inlineStr"/>
-    </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="17" t="inlineStr">
-        <is>
-          <t>CAMPOS OBRIGATÓRIOS (fundo rosa)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Nome Completo: Nome completo do funcionário.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Cargo / Função: Função que o funcionário exerce na empresa.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Custo por Hora (R$): Valor em reais por hora trabalhada.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Horas por Dia Útil: Padrão = 9h. Aceita valores entre 1 e 24.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Ativo (SIM/NÃO): SIM = funcionário ativo, NÃO = inativo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="6" customHeight="1">
-      <c r="A9" s="16" t="inlineStr"/>
-    </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="19" t="inlineStr">
-        <is>
-          <t>CAMPOS OPCIONAIS (fundo azul)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • E-mail: E-mail profissional do funcionário.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Telefone: Formato sugerido: (37) 99999-9999</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="6" customHeight="1">
-      <c r="A13" s="16" t="inlineStr"/>
-    </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="20" t="inlineStr">
-        <is>
-          <t>COMO IMPORTAR</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  1. Preencha os dados a partir da linha 5 (não altere as linhas 1–4).</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  2. Salve no formato .xlsx</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  3. No sistema → Funcionários → botão 'Importar Excel'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  4. Revise a pré-visualização e confirme a importação.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="6" customHeight="1">
-      <c r="A19" s="16" t="inlineStr"/>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="21" t="inlineStr">
-        <is>
-          <t>OBSERVAÇÕES</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Não altere os cabeçalhos (linha 3) nem a estrutura das colunas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • A linha verde (linha 4) é apenas exemplo — não será importada.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Máximo de 100 funcionários por importação.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Consulte a aba 'Cargos de Referência' para sugestões de função.</t>
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>Cargos / Funções Sugeridos</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Cargo / Função</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="inlineStr">
+        <is>
+          <t>Setor Típico</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>Engenheiro Eletricista</t>
+        </is>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>Engenharia Elétrica</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>Engenheiro de Automação</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>Engenharia de Automação</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>Técnico em Automação</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>Engenharia de Automação</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>Programador CLP</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>Engenharia de Automação</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>Programador SCADA</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>Engenharia de Software</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>Projetista Elétrico</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>Projetos</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>Eletricista Industrial</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>Montagem de Campo</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>Eletricista Instalador</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>Montagem de Campo</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>Auxiliar Elétrico</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>Montagem de Campo</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>Montador de Painel</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>Montagem de Painel</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>Técnico de Campo</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>Montagem de Campo</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>Supervisor de Obras</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>Montagem de Campo</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>Encarregado de Obras</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>Montagem de Campo</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>Assistente Técnico</t>
+        </is>
+      </c>
+      <c r="B16" s="14" t="inlineStr">
+        <is>
+          <t>Suporte Técnico</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>Gerente de Projetos</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>Administrativo</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>Coordenador de Automação</t>
+        </is>
+      </c>
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>Engenharia de Automação</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>